<commit_message>
Made changes to part 4 code and completed part 5
</commit_message>
<xml_diff>
--- a/Lab4_ADC/lab4.xlsx
+++ b/Lab4_ADC/lab4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uoa-my.sharepoint.com/personal/mden116_uoa_auckland_ac_nz/Documents/Documents/Assignments_exams/part 2/ee209/EE209Labs/Lab4_ADC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="8_{4608927A-F8E1-47F5-B52E-1D221F88EBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F9E09D4C-DCE6-49E1-9F05-A5C91656B425}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{4608927A-F8E1-47F5-B52E-1D221F88EBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3715B514-6D4A-4FCB-9F51-0D5363D0BB43}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5DD0FFD9-16EF-4DC0-9893-E6A77CC9477E}"/>
   </bookViews>
@@ -36,6 +36,10 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -154,7 +158,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-US"/>
+          <a:endParaRPr lang="en-NZ"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -204,121 +208,121 @@
                   <c:v>849</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>854</c:v>
+                  <c:v>576</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2958</c:v>
+                  <c:v>1606</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4472</c:v>
+                  <c:v>3247</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3476</c:v>
+                  <c:v>4384</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1240</c:v>
+                  <c:v>4243</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>605</c:v>
+                  <c:v>2915</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2382</c:v>
+                  <c:v>1308</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>4306</c:v>
+                  <c:v>512</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3935</c:v>
+                  <c:v>1069</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1733</c:v>
+                  <c:v>2597</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>507</c:v>
+                  <c:v>4057</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1816</c:v>
+                  <c:v>4458</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3999</c:v>
+                  <c:v>3530</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>4272</c:v>
+                  <c:v>1899</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>2294</c:v>
+                  <c:v>673</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>576</c:v>
+                  <c:v>693</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>1303</c:v>
+                  <c:v>1938</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3554</c:v>
+                  <c:v>3564</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>4458</c:v>
+                  <c:v>4467</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2871</c:v>
+                  <c:v>4033</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>810</c:v>
+                  <c:v>2558</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>898</c:v>
+                  <c:v>1035</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>3027</c:v>
+                  <c:v>517</c:v>
                 </c:pt>
                 <c:pt idx="24">
+                  <c:v>1337</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>2954</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>4257</c:v>
+                </c:pt>
+                <c:pt idx="27">
+                  <c:v>4365</c:v>
+                </c:pt>
+                <c:pt idx="28">
+                  <c:v>3208</c:v>
+                </c:pt>
+                <c:pt idx="29">
+                  <c:v>1567</c:v>
+                </c:pt>
+                <c:pt idx="30">
+                  <c:v>556</c:v>
+                </c:pt>
+                <c:pt idx="31">
+                  <c:v>869</c:v>
+                </c:pt>
+                <c:pt idx="32">
+                  <c:v>2290</c:v>
+                </c:pt>
+                <c:pt idx="33">
+                  <c:v>3847</c:v>
+                </c:pt>
+                <c:pt idx="34">
                   <c:v>4487</c:v>
                 </c:pt>
-                <c:pt idx="25">
-                  <c:v>3413</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>1186</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>625</c:v>
-                </c:pt>
-                <c:pt idx="28">
-                  <c:v>2451</c:v>
-                </c:pt>
-                <c:pt idx="29">
-                  <c:v>4335</c:v>
-                </c:pt>
-                <c:pt idx="30">
-                  <c:v>3881</c:v>
-                </c:pt>
-                <c:pt idx="31">
-                  <c:v>1669</c:v>
-                </c:pt>
-                <c:pt idx="32">
-                  <c:v>512</c:v>
-                </c:pt>
-                <c:pt idx="33">
-                  <c:v>1879</c:v>
-                </c:pt>
-                <c:pt idx="34">
-                  <c:v>4042</c:v>
-                </c:pt>
                 <c:pt idx="35">
-                  <c:v>4243</c:v>
+                  <c:v>3779</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>2221</c:v>
+                  <c:v>2197</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>556</c:v>
+                  <c:v>825</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>1362</c:v>
+                  <c:v>590</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>3618</c:v>
+                  <c:v>1650</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -367,124 +371,124 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="40"/>
                 <c:pt idx="0">
-                  <c:v>1635</c:v>
+                  <c:v>1567</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2651</c:v>
+                  <c:v>2138</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3476</c:v>
+                  <c:v>2958</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3056</c:v>
+                  <c:v>3466</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1933</c:v>
+                  <c:v>3320</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1528</c:v>
+                  <c:v>2612</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2363</c:v>
+                  <c:v>1831</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>3369</c:v>
+                  <c:v>1503</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>3271</c:v>
+                  <c:v>1855</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>2192</c:v>
+                  <c:v>2641</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1503</c:v>
+                  <c:v>3334</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2084</c:v>
+                  <c:v>3457</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3193</c:v>
+                  <c:v>2929</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3422</c:v>
+                  <c:v>2109</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>2475</c:v>
+                  <c:v>1557</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>1567</c:v>
+                  <c:v>1640</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>1840</c:v>
+                  <c:v>2309</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>2958</c:v>
+                  <c:v>3110</c:v>
                 </c:pt>
                 <c:pt idx="18">
                   <c:v>3491</c:v>
                 </c:pt>
                 <c:pt idx="19">
+                  <c:v>3203</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>2431</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1708</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>1523</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>2001</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>2817</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>3417</c:v>
+                </c:pt>
+                <c:pt idx="26">
+                  <c:v>3398</c:v>
+                </c:pt>
+                <c:pt idx="27">
                   <c:v>2763</c:v>
                 </c:pt>
-                <c:pt idx="20">
-                  <c:v>1699</c:v>
-                </c:pt>
-                <c:pt idx="21">
-                  <c:v>1655</c:v>
-                </c:pt>
-                <c:pt idx="22">
-                  <c:v>2685</c:v>
-                </c:pt>
-                <c:pt idx="23">
-                  <c:v>3481</c:v>
-                </c:pt>
-                <c:pt idx="24">
-                  <c:v>3027</c:v>
-                </c:pt>
-                <c:pt idx="25">
-                  <c:v>1904</c:v>
-                </c:pt>
-                <c:pt idx="26">
-                  <c:v>1538</c:v>
-                </c:pt>
-                <c:pt idx="27">
-                  <c:v>2397</c:v>
-                </c:pt>
                 <c:pt idx="28">
-                  <c:v>3383</c:v>
+                  <c:v>1953</c:v>
                 </c:pt>
                 <c:pt idx="29">
-                  <c:v>3247</c:v>
+                  <c:v>1508</c:v>
                 </c:pt>
                 <c:pt idx="30">
-                  <c:v>2158</c:v>
+                  <c:v>1743</c:v>
                 </c:pt>
                 <c:pt idx="31">
-                  <c:v>1503</c:v>
+                  <c:v>2490</c:v>
                 </c:pt>
                 <c:pt idx="32">
-                  <c:v>2119</c:v>
+                  <c:v>3242</c:v>
                 </c:pt>
                 <c:pt idx="33">
-                  <c:v>3217</c:v>
+                  <c:v>3486</c:v>
                 </c:pt>
                 <c:pt idx="34">
-                  <c:v>3408</c:v>
+                  <c:v>3061</c:v>
                 </c:pt>
                 <c:pt idx="35">
-                  <c:v>2441</c:v>
+                  <c:v>2255</c:v>
                 </c:pt>
                 <c:pt idx="36">
-                  <c:v>1552</c:v>
+                  <c:v>1611</c:v>
                 </c:pt>
                 <c:pt idx="37">
-                  <c:v>1870</c:v>
+                  <c:v>1577</c:v>
                 </c:pt>
                 <c:pt idx="38">
-                  <c:v>2993</c:v>
+                  <c:v>2163</c:v>
                 </c:pt>
                 <c:pt idx="39">
-                  <c:v>3486</c:v>
+                  <c:v>2983</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -572,7 +576,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-US"/>
+              <a:endParaRPr lang="en-NZ"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1399,6 +1403,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1726,148 +1734,148 @@
         <v>849</v>
       </c>
       <c r="B1">
-        <v>1635</v>
+        <v>1567</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2">
-        <v>854</v>
+        <v>576</v>
       </c>
       <c r="B2">
-        <v>2651</v>
+        <v>2138</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3">
+        <v>1606</v>
+      </c>
+      <c r="B3">
         <v>2958</v>
-      </c>
-      <c r="B3">
-        <v>3476</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>4472</v>
+        <v>3247</v>
       </c>
       <c r="B4">
-        <v>3056</v>
+        <v>3466</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>3476</v>
+        <v>4384</v>
       </c>
       <c r="B5">
-        <v>1933</v>
+        <v>3320</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>1240</v>
+        <v>4243</v>
       </c>
       <c r="B6">
-        <v>1528</v>
+        <v>2612</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>605</v>
+        <v>2915</v>
       </c>
       <c r="B7">
-        <v>2363</v>
+        <v>1831</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>2382</v>
+        <v>1308</v>
       </c>
       <c r="B8">
-        <v>3369</v>
+        <v>1503</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>4306</v>
+        <v>512</v>
       </c>
       <c r="B9">
-        <v>3271</v>
+        <v>1855</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>3935</v>
+        <v>1069</v>
       </c>
       <c r="B10">
-        <v>2192</v>
+        <v>2641</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>1733</v>
+        <v>2597</v>
       </c>
       <c r="B11">
-        <v>1503</v>
+        <v>3334</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>507</v>
+        <v>4057</v>
       </c>
       <c r="B12">
-        <v>2084</v>
+        <v>3457</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>1816</v>
+        <v>4458</v>
       </c>
       <c r="B13">
-        <v>3193</v>
+        <v>2929</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>3999</v>
+        <v>3530</v>
       </c>
       <c r="B14">
-        <v>3422</v>
+        <v>2109</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>4272</v>
+        <v>1899</v>
       </c>
       <c r="B15">
-        <v>2475</v>
+        <v>1557</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>2294</v>
+        <v>673</v>
       </c>
       <c r="B16">
-        <v>1567</v>
+        <v>1640</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>576</v>
+        <v>693</v>
       </c>
       <c r="B17">
-        <v>1840</v>
+        <v>2309</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>1303</v>
+        <v>1938</v>
       </c>
       <c r="B18">
-        <v>2958</v>
+        <v>3110</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>3554</v>
+        <v>3564</v>
       </c>
       <c r="B19">
         <v>3491</v>
@@ -1875,174 +1883,175 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>4458</v>
+        <v>4467</v>
       </c>
       <c r="B20">
-        <v>2763</v>
+        <v>3203</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>2871</v>
+        <v>4033</v>
       </c>
       <c r="B21">
-        <v>1699</v>
+        <v>2431</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>810</v>
+        <v>2558</v>
       </c>
       <c r="B22">
-        <v>1655</v>
+        <v>1708</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>898</v>
+        <v>1035</v>
       </c>
       <c r="B23">
-        <v>2685</v>
+        <v>1523</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>3027</v>
+        <v>517</v>
       </c>
       <c r="B24">
-        <v>3481</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>4487</v>
+        <v>1337</v>
       </c>
       <c r="B25">
-        <v>3027</v>
+        <v>2817</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>3413</v>
+        <v>2954</v>
       </c>
       <c r="B26">
-        <v>1904</v>
+        <v>3417</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>1186</v>
+        <v>4257</v>
       </c>
       <c r="B27">
-        <v>1538</v>
+        <v>3398</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>625</v>
+        <v>4365</v>
       </c>
       <c r="B28">
-        <v>2397</v>
+        <v>2763</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>2451</v>
+        <v>3208</v>
       </c>
       <c r="B29">
-        <v>3383</v>
+        <v>1953</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>4335</v>
+        <v>1567</v>
       </c>
       <c r="B30">
-        <v>3247</v>
+        <v>1508</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>3881</v>
+        <v>556</v>
       </c>
       <c r="B31">
-        <v>2158</v>
+        <v>1743</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>1669</v>
+        <v>869</v>
       </c>
       <c r="B32">
-        <v>1503</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>512</v>
+        <v>2290</v>
       </c>
       <c r="B33">
-        <v>2119</v>
+        <v>3242</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>1879</v>
+        <v>3847</v>
       </c>
       <c r="B34">
-        <v>3217</v>
+        <v>3486</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>4042</v>
+        <v>4487</v>
       </c>
       <c r="B35">
-        <v>3408</v>
+        <v>3061</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>4243</v>
+        <v>3779</v>
       </c>
       <c r="B36">
-        <v>2441</v>
+        <v>2255</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>2221</v>
+        <v>2197</v>
       </c>
       <c r="B37">
-        <v>1552</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>556</v>
+        <v>825</v>
       </c>
       <c r="B38">
-        <v>1870</v>
+        <v>1577</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>1362</v>
+        <v>590</v>
       </c>
       <c r="B39">
-        <v>2993</v>
+        <v>2163</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>3618</v>
+        <v>1650</v>
       </c>
       <c r="B40">
-        <v>3486</v>
+        <v>2983</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>